<commit_message>
Arabic-only labels and definitions in the simple entry template
KPI names with APEX/OPD and three English definitions get Arabic labels
(KPI_ARABIC_LABELS in index.html); the importer accepts those labels too.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TCe2cBGNmZWP82GSjm6P4E
</commit_message>
<xml_diff>
--- a/templates/APH_KPI_Simple_2026.xlsx
+++ b/templates/APH_KPI_Simple_2026.xlsx
@@ -1102,12 +1102,12 @@
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>عدد مراجعي العيادات (APEX)</t>
+          <t>عدد مراجعي العيادات (نظام أبكس)</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>المرضى الذين لم يحضروا للمواعيد (APEX)</t>
+          <t>المرضى الذين لم يحضروا للمواعيد (نظام أبكس)</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="AJ3" s="5" t="inlineStr">
         <is>
-          <t>تجربة المريض - OPD</t>
+          <t>تجربة المريض - العيادات الخارجية</t>
         </is>
       </c>
       <c r="AK3" s="5" t="inlineStr">
@@ -17792,7 +17792,7 @@
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
-          <t>Hospital Readmission Rate same diagnosis within 30 days (%)</t>
+          <t>نسبة المرضى الذين أُعيد تنويمهم خلال 30 يوماً بنفس التشخيص من إجمالي المخرَّجين أحياء (%)</t>
         </is>
       </c>
     </row>
@@ -17832,7 +17832,7 @@
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>Hospital Readmission Rate same diagnosis within 30 days (%)</t>
+          <t>نسبة المرضى الذين أُعيد تنويمهم خلال 30 يوماً بنفس التشخيص من إجمالي المخرَّجين أحياء (%)</t>
         </is>
       </c>
     </row>
@@ -18120,14 +18120,14 @@
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>Hospital Revisit Rate same diagnosis within 72 days (%) [label says days; title says hours]</t>
+          <t>نسبة العودة غير المخطط لها للطوارئ خلال 72 ساعة بنفس التشخيص من إجمالي مراجعي الطوارئ (%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>عدد مراجعي العيادات (APEX)</t>
+          <t>عدد مراجعي العيادات (نظام أبكس)</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
@@ -18163,7 +18163,7 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>المرضى الذين لم يحضروا للمواعيد (APEX)</t>
+          <t>المرضى الذين لم يحضروا للمواعيد (نظام أبكس)</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -18697,7 +18697,7 @@
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>تجربة المريض - OPD</t>
+          <t>تجربة المريض - العيادات الخارجية</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Add nursing KPIs to the platform and template; cap achievement at 100% (v4.5)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuVEaC2eFdeXs882mV4a9X
</commit_message>
<xml_diff>
--- a/templates/APH_KPI_Simple_2026.xlsx
+++ b/templates/APH_KPI_Simple_2026.xlsx
@@ -995,7 +995,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:AG32"/>
+  <dimension ref="A1:AG36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -2432,10 +2432,198 @@
       <c r="AF32" s="9"/>
       <c r="AG32" s="11"/>
     </row>
+    <row r="33" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="11"/>
+    </row>
+    <row r="34" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="11"/>
+    </row>
+    <row r="35" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="11"/>
+    </row>
+    <row r="36" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AG32" xr:uid="{00000000-0002-0000-0900-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AG32 D33:AH36" xr:uid="{00000000-0002-0000-0900-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -2445,7 +2633,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:AH32"/>
+  <dimension ref="A1:AH36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -3918,10 +4106,202 @@
       <c r="AG32" s="9"/>
       <c r="AH32" s="11"/>
     </row>
+    <row r="33" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="9"/>
+      <c r="AH33" s="11"/>
+    </row>
+    <row r="34" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="9"/>
+      <c r="AH34" s="11"/>
+    </row>
+    <row r="35" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="9"/>
+      <c r="AH35" s="11"/>
+    </row>
+    <row r="36" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="9"/>
+      <c r="AH36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32" xr:uid="{00000000-0002-0000-0A00-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32 D33:AH36" xr:uid="{00000000-0002-0000-0A00-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -3932,7 +4312,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:AG32"/>
+  <dimension ref="A1:AG36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -5369,10 +5749,198 @@
       <c r="AF32" s="9"/>
       <c r="AG32" s="11"/>
     </row>
+    <row r="33" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="11"/>
+    </row>
+    <row r="34" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="11"/>
+    </row>
+    <row r="35" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="11"/>
+    </row>
+    <row r="36" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AG32" xr:uid="{00000000-0002-0000-0B00-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AG32 D33:AH36" xr:uid="{00000000-0002-0000-0B00-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -5382,7 +5950,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:AH32"/>
+  <dimension ref="A1:AH36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -6855,10 +7423,202 @@
       <c r="AG32" s="9"/>
       <c r="AH32" s="11"/>
     </row>
+    <row r="33" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="9"/>
+      <c r="AH33" s="11"/>
+    </row>
+    <row r="34" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="9"/>
+      <c r="AH34" s="11"/>
+    </row>
+    <row r="35" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="9"/>
+      <c r="AH35" s="11"/>
+    </row>
+    <row r="36" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="9"/>
+      <c r="AH36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32" xr:uid="{00000000-0002-0000-0C00-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32 D33:AH36" xr:uid="{00000000-0002-0000-0C00-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -7616,16 +8376,162 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H32" s="14"/>
-    </row>
-    <row r="33" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H33" s="14"/>
-    </row>
-    <row r="34" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H34" s="14"/>
-    </row>
-    <row r="35" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H35" s="14"/>
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>شهري</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>اخر يوم في الشهر</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>القيمة</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G32" s="13">
+        <v>0</v>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>عدد المرضى الذين أصيبوا بقرحة فراش أثناء التنويم ÷ إجمالي المرضى المنومين × 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>شهري</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>اخر يوم في الشهر</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>القيمة</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>لكل 1000</t>
+        </is>
+      </c>
+      <c r="G33" s="13">
+        <v>0</v>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>عدد حالات سقوط المرضى أثناء التنويم (مع إصابة أو بدونها) ÷ إجمالي المرضى المنومين (الأسرّة المشغولة) × 1000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>شهري</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>اخر يوم في الشهر</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>القيمة</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G34" s="13">
+        <v>0</v>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>عدد محاولات الانتحار الفعلية أثناء التنويم ÷ إجمالي المرضى المنومين × 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>شهري</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>اخر يوم في الشهر</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>القيمة</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>عدد</t>
+        </is>
+      </c>
+      <c r="G35" s="13"/>
+      <c r="H35" s="10" t="inlineStr">
+        <is>
+          <t>إجمالي نداءات Mr. Strong في جميع الأقسام خلال الشهر.</t>
+        </is>
+      </c>
     </row>
     <row r="36" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H36" s="14"/>
@@ -7733,7 +8639,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AH32"/>
+  <dimension ref="A1:AH36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -9205,10 +10111,202 @@
       <c r="AF32" s="9"/>
       <c r="AG32" s="9"/>
     </row>
+    <row r="33" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="9"/>
+      <c r="AH33" s="11"/>
+    </row>
+    <row r="34" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="9"/>
+      <c r="AH34" s="11"/>
+    </row>
+    <row r="35" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="9"/>
+      <c r="AH35" s="11"/>
+    </row>
+    <row r="36" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="9"/>
+      <c r="AH36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="AH3:AH31 D3:AG32" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="AH3:AH31 D3:AG32 D33:AH36" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -9218,7 +10316,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AE32"/>
+  <dimension ref="A1:AE36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -10582,10 +11680,190 @@
       <c r="AC32" s="9"/>
       <c r="AD32" s="9"/>
     </row>
+    <row r="33" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="11"/>
+    </row>
+    <row r="34" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="11"/>
+    </row>
+    <row r="35" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="11"/>
+    </row>
+    <row r="36" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="AE3:AE31 D3:AD32" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="AE3:AE31 D3:AD32 D33:AH36" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -10595,7 +11873,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:AH32"/>
+  <dimension ref="A1:AH36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -12068,10 +13346,202 @@
       <c r="AG32" s="9"/>
       <c r="AH32" s="11"/>
     </row>
+    <row r="33" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="9"/>
+      <c r="AH33" s="11"/>
+    </row>
+    <row r="34" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="9"/>
+      <c r="AH34" s="11"/>
+    </row>
+    <row r="35" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="9"/>
+      <c r="AH35" s="11"/>
+    </row>
+    <row r="36" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="9"/>
+      <c r="AH36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32 D33:AH36" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -12081,7 +13551,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:AG32"/>
+  <dimension ref="A1:AG36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -13518,10 +14988,198 @@
       <c r="AF32" s="9"/>
       <c r="AG32" s="11"/>
     </row>
+    <row r="33" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="11"/>
+    </row>
+    <row r="34" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="11"/>
+    </row>
+    <row r="35" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="11"/>
+    </row>
+    <row r="36" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AG32" xr:uid="{00000000-0002-0000-0400-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AG32 D33:AH36" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -13531,7 +15189,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:AH32"/>
+  <dimension ref="A1:AH36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -15004,10 +16662,202 @@
       <c r="AG32" s="9"/>
       <c r="AH32" s="11"/>
     </row>
+    <row r="33" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="9"/>
+      <c r="AH33" s="11"/>
+    </row>
+    <row r="34" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="9"/>
+      <c r="AH34" s="11"/>
+    </row>
+    <row r="35" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="9"/>
+      <c r="AH35" s="11"/>
+    </row>
+    <row r="36" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="9"/>
+      <c r="AH36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32" xr:uid="{00000000-0002-0000-0500-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32 D33:AH36" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -15017,7 +16867,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:AG32"/>
+  <dimension ref="A1:AG36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -16454,10 +18304,198 @@
       <c r="AF32" s="9"/>
       <c r="AG32" s="11"/>
     </row>
+    <row r="33" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="11"/>
+    </row>
+    <row r="34" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="11"/>
+    </row>
+    <row r="35" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="11"/>
+    </row>
+    <row r="36" spans="1:33" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AG32" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AG32 D33:AH36" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -16467,7 +18505,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:AH32"/>
+  <dimension ref="A1:AH36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -17940,10 +19978,202 @@
       <c r="AG32" s="9"/>
       <c r="AH32" s="11"/>
     </row>
+    <row r="33" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="9"/>
+      <c r="AH33" s="11"/>
+    </row>
+    <row r="34" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="9"/>
+      <c r="AH34" s="11"/>
+    </row>
+    <row r="35" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="9"/>
+      <c r="AH35" s="11"/>
+    </row>
+    <row r="36" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="9"/>
+      <c r="AH36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32" xr:uid="{00000000-0002-0000-0700-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32 D33:AH36" xr:uid="{00000000-0002-0000-0700-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -17953,7 +20183,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:AH32"/>
+  <dimension ref="A1:AH36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" hidden="1" customWidth="1"/>
@@ -19426,10 +21656,202 @@
       <c r="AG32" s="9"/>
       <c r="AH32" s="11"/>
     </row>
+    <row r="33" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NURS_PRESSURE_ULCER</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>قرح الفراش المكتسبة في المستشفى</t>
+        </is>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+      <c r="Y33" s="9"/>
+      <c r="Z33" s="9"/>
+      <c r="AA33" s="9"/>
+      <c r="AB33" s="9"/>
+      <c r="AC33" s="9"/>
+      <c r="AD33" s="9"/>
+      <c r="AE33" s="9"/>
+      <c r="AF33" s="9"/>
+      <c r="AG33" s="9"/>
+      <c r="AH33" s="11"/>
+    </row>
+    <row r="34" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NURS_PATIENT_FALL</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>سقوط المرضى</t>
+        </is>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="9"/>
+      <c r="AA34" s="9"/>
+      <c r="AB34" s="9"/>
+      <c r="AC34" s="9"/>
+      <c r="AD34" s="9"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="9"/>
+      <c r="AG34" s="9"/>
+      <c r="AH34" s="11"/>
+    </row>
+    <row r="35" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NURS_ATTEMPTED_SUICIDE</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>محاولات الانتحار</t>
+        </is>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="9"/>
+      <c r="AH35" s="11"/>
+    </row>
+    <row r="36" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NURS_MR_STRONG</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>إدارة التمريض</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>نداءات Mr. Strong</t>
+        </is>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="9"/>
+      <c r="AH36" s="11"/>
+    </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32" xr:uid="{00000000-0002-0000-0800-000000000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اكتب رقماً فقط (صفر أو أكثر) بدون رموز أو نص." sqref="D3:AH32 D33:AH36" xr:uid="{00000000-0002-0000-0800-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Nursing readings go on the 1st of the following month in the template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuVEaC2eFdeXs882mV4a9X
</commit_message>
<xml_diff>
--- a/templates/APH_KPI_Simple_2026.xlsx
+++ b/templates/APH_KPI_Simple_2026.xlsx
@@ -2448,7 +2448,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2477,7 +2477,7 @@
       <c r="AD33" s="9"/>
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
-      <c r="AG33" s="11"/>
+      <c r="AG33" s="9"/>
     </row>
     <row r="34" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -2495,7 +2495,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2524,7 +2524,7 @@
       <c r="AD34" s="9"/>
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
-      <c r="AG34" s="11"/>
+      <c r="AG34" s="9"/>
     </row>
     <row r="35" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -2542,7 +2542,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2571,7 +2571,7 @@
       <c r="AD35" s="9"/>
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
-      <c r="AG35" s="11"/>
+      <c r="AG35" s="9"/>
     </row>
     <row r="36" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -2589,7 +2589,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2618,7 +2618,7 @@
       <c r="AD36" s="9"/>
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
-      <c r="AG36" s="11"/>
+      <c r="AG36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -4122,7 +4122,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -4152,7 +4152,7 @@
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
       <c r="AG33" s="9"/>
-      <c r="AH33" s="11"/>
+      <c r="AH33" s="9"/>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -4170,7 +4170,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -4200,7 +4200,7 @@
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
       <c r="AG34" s="9"/>
-      <c r="AH34" s="11"/>
+      <c r="AH34" s="9"/>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -4218,7 +4218,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -4248,7 +4248,7 @@
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
       <c r="AG35" s="9"/>
-      <c r="AH35" s="11"/>
+      <c r="AH35" s="9"/>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -4266,7 +4266,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -4296,7 +4296,7 @@
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
       <c r="AG36" s="9"/>
-      <c r="AH36" s="11"/>
+      <c r="AH36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -5765,7 +5765,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -5794,7 +5794,7 @@
       <c r="AD33" s="9"/>
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
-      <c r="AG33" s="11"/>
+      <c r="AG33" s="9"/>
     </row>
     <row r="34" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -5812,7 +5812,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -5841,7 +5841,7 @@
       <c r="AD34" s="9"/>
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
-      <c r="AG34" s="11"/>
+      <c r="AG34" s="9"/>
     </row>
     <row r="35" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -5859,7 +5859,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -5888,7 +5888,7 @@
       <c r="AD35" s="9"/>
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
-      <c r="AG35" s="11"/>
+      <c r="AG35" s="9"/>
     </row>
     <row r="36" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -5906,7 +5906,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -5935,7 +5935,7 @@
       <c r="AD36" s="9"/>
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
-      <c r="AG36" s="11"/>
+      <c r="AG36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -7439,7 +7439,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -7469,7 +7469,7 @@
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
       <c r="AG33" s="9"/>
-      <c r="AH33" s="11"/>
+      <c r="AH33" s="9"/>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -7487,7 +7487,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -7517,7 +7517,7 @@
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
       <c r="AG34" s="9"/>
-      <c r="AH34" s="11"/>
+      <c r="AH34" s="9"/>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -7535,7 +7535,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -7565,7 +7565,7 @@
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
       <c r="AG35" s="9"/>
-      <c r="AH35" s="11"/>
+      <c r="AH35" s="9"/>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -7583,7 +7583,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -7613,7 +7613,7 @@
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
       <c r="AG36" s="9"/>
-      <c r="AH36" s="11"/>
+      <c r="AH36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -8393,7 +8393,7 @@
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>اخر يوم في الشهر</t>
+          <t>أول يوم من الشهر التالي</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
@@ -8433,7 +8433,7 @@
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>اخر يوم في الشهر</t>
+          <t>أول يوم من الشهر التالي</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>اخر يوم في الشهر</t>
+          <t>أول يوم من الشهر التالي</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
@@ -8513,7 +8513,7 @@
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>اخر يوم في الشهر</t>
+          <t>أول يوم من الشهر التالي</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -10127,7 +10127,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -10157,7 +10157,7 @@
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
       <c r="AG33" s="9"/>
-      <c r="AH33" s="11"/>
+      <c r="AH33" s="9"/>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -10175,7 +10175,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -10205,7 +10205,7 @@
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
       <c r="AG34" s="9"/>
-      <c r="AH34" s="11"/>
+      <c r="AH34" s="9"/>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -10223,7 +10223,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -10253,7 +10253,7 @@
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
       <c r="AG35" s="9"/>
-      <c r="AH35" s="11"/>
+      <c r="AH35" s="9"/>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -10271,7 +10271,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -10301,7 +10301,7 @@
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
       <c r="AG36" s="9"/>
-      <c r="AH36" s="11"/>
+      <c r="AH36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -11696,7 +11696,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -11723,7 +11723,7 @@
       <c r="AB33" s="9"/>
       <c r="AC33" s="9"/>
       <c r="AD33" s="9"/>
-      <c r="AE33" s="11"/>
+      <c r="AE33" s="9"/>
     </row>
     <row r="34" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -11741,7 +11741,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -11768,7 +11768,7 @@
       <c r="AB34" s="9"/>
       <c r="AC34" s="9"/>
       <c r="AD34" s="9"/>
-      <c r="AE34" s="11"/>
+      <c r="AE34" s="9"/>
     </row>
     <row r="35" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -11786,7 +11786,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -11813,7 +11813,7 @@
       <c r="AB35" s="9"/>
       <c r="AC35" s="9"/>
       <c r="AD35" s="9"/>
-      <c r="AE35" s="11"/>
+      <c r="AE35" s="9"/>
     </row>
     <row r="36" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -11831,7 +11831,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -11858,7 +11858,7 @@
       <c r="AB36" s="9"/>
       <c r="AC36" s="9"/>
       <c r="AD36" s="9"/>
-      <c r="AE36" s="11"/>
+      <c r="AE36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -13362,7 +13362,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -13392,7 +13392,7 @@
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
       <c r="AG33" s="9"/>
-      <c r="AH33" s="11"/>
+      <c r="AH33" s="9"/>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -13410,7 +13410,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -13440,7 +13440,7 @@
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
       <c r="AG34" s="9"/>
-      <c r="AH34" s="11"/>
+      <c r="AH34" s="9"/>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -13458,7 +13458,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -13488,7 +13488,7 @@
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
       <c r="AG35" s="9"/>
-      <c r="AH35" s="11"/>
+      <c r="AH35" s="9"/>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -13506,7 +13506,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -13536,7 +13536,7 @@
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
       <c r="AG36" s="9"/>
-      <c r="AH36" s="11"/>
+      <c r="AH36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -15004,7 +15004,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -15033,7 +15033,7 @@
       <c r="AD33" s="9"/>
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
-      <c r="AG33" s="11"/>
+      <c r="AG33" s="9"/>
     </row>
     <row r="34" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -15051,7 +15051,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -15080,7 +15080,7 @@
       <c r="AD34" s="9"/>
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
-      <c r="AG34" s="11"/>
+      <c r="AG34" s="9"/>
     </row>
     <row r="35" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -15098,7 +15098,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -15127,7 +15127,7 @@
       <c r="AD35" s="9"/>
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
-      <c r="AG35" s="11"/>
+      <c r="AG35" s="9"/>
     </row>
     <row r="36" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -15145,7 +15145,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -15174,7 +15174,7 @@
       <c r="AD36" s="9"/>
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
-      <c r="AG36" s="11"/>
+      <c r="AG36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -16678,7 +16678,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -16708,7 +16708,7 @@
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
       <c r="AG33" s="9"/>
-      <c r="AH33" s="11"/>
+      <c r="AH33" s="9"/>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -16726,7 +16726,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -16756,7 +16756,7 @@
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
       <c r="AG34" s="9"/>
-      <c r="AH34" s="11"/>
+      <c r="AH34" s="9"/>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -16774,7 +16774,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -16804,7 +16804,7 @@
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
       <c r="AG35" s="9"/>
-      <c r="AH35" s="11"/>
+      <c r="AH35" s="9"/>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -16822,7 +16822,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -16852,7 +16852,7 @@
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
       <c r="AG36" s="9"/>
-      <c r="AH36" s="11"/>
+      <c r="AH36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -18320,7 +18320,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -18349,7 +18349,7 @@
       <c r="AD33" s="9"/>
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
-      <c r="AG33" s="11"/>
+      <c r="AG33" s="9"/>
     </row>
     <row r="34" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -18367,7 +18367,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -18396,7 +18396,7 @@
       <c r="AD34" s="9"/>
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
-      <c r="AG34" s="11"/>
+      <c r="AG34" s="9"/>
     </row>
     <row r="35" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -18414,7 +18414,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -18443,7 +18443,7 @@
       <c r="AD35" s="9"/>
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
-      <c r="AG35" s="11"/>
+      <c r="AG35" s="9"/>
     </row>
     <row r="36" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -18461,7 +18461,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -18490,7 +18490,7 @@
       <c r="AD36" s="9"/>
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
-      <c r="AG36" s="11"/>
+      <c r="AG36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -19994,7 +19994,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -20024,7 +20024,7 @@
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
       <c r="AG33" s="9"/>
-      <c r="AH33" s="11"/>
+      <c r="AH33" s="9"/>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -20042,7 +20042,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -20072,7 +20072,7 @@
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
       <c r="AG34" s="9"/>
-      <c r="AH34" s="11"/>
+      <c r="AH34" s="9"/>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -20090,7 +20090,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -20120,7 +20120,7 @@
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
       <c r="AG35" s="9"/>
-      <c r="AH35" s="11"/>
+      <c r="AH35" s="9"/>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -20138,7 +20138,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -20168,7 +20168,7 @@
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
       <c r="AG36" s="9"/>
-      <c r="AH36" s="11"/>
+      <c r="AH36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>
@@ -21672,7 +21672,7 @@
           <t>قرح الفراش المكتسبة في المستشفى</t>
         </is>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="11"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -21702,7 +21702,7 @@
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
       <c r="AG33" s="9"/>
-      <c r="AH33" s="11"/>
+      <c r="AH33" s="9"/>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A34" t="inlineStr">
@@ -21720,7 +21720,7 @@
           <t>سقوط المرضى</t>
         </is>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="11"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -21750,7 +21750,7 @@
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
       <c r="AG34" s="9"/>
-      <c r="AH34" s="11"/>
+      <c r="AH34" s="9"/>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A35" t="inlineStr">
@@ -21768,7 +21768,7 @@
           <t>محاولات الانتحار</t>
         </is>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="11"/>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -21798,7 +21798,7 @@
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
       <c r="AG35" s="9"/>
-      <c r="AH35" s="11"/>
+      <c r="AH35" s="9"/>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A36" t="inlineStr">
@@ -21816,7 +21816,7 @@
           <t>نداءات Mr. Strong</t>
         </is>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="11"/>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -21846,7 +21846,7 @@
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
       <c r="AG36" s="9"/>
-      <c r="AH36" s="11"/>
+      <c r="AH36" s="9"/>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0"/>

</xml_diff>